<commit_message>
use correct FT jobs
</commit_message>
<xml_diff>
--- a/eval/results/evaluation_metrics_by_qid_full150.xlsx
+++ b/eval/results/evaluation_metrics_by_qid_full150.xlsx
@@ -501,25 +501,25 @@
         <v>150</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.86</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9263157894736842</v>
       </c>
       <c r="D2" t="n">
         <v>0.8627450980392157</v>
       </c>
       <c r="E2" t="n">
-        <v>0.888888888888889</v>
+        <v>0.8934010152284264</v>
       </c>
       <c r="F2" t="n">
         <v>88</v>
       </c>
       <c r="G2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2" t="n">
         <v>14</v>
@@ -548,19 +548,19 @@
         <v>150</v>
       </c>
       <c r="B3" t="n">
-        <v>0.92</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9215686274509803</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9306930693069307</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G3" t="n">
         <v>42</v>
@@ -569,7 +569,7 @@
         <v>6</v>
       </c>
       <c r="I3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -642,19 +642,19 @@
         <v>150</v>
       </c>
       <c r="B5" t="n">
-        <v>0.76</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9125</v>
+        <v>0.9146341463414634</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7156862745098039</v>
+        <v>0.7352941176470589</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8021978021978022</v>
+        <v>0.8152173913043479</v>
       </c>
       <c r="F5" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
         <v>41</v>
@@ -663,7 +663,7 @@
         <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -689,19 +689,19 @@
         <v>150</v>
       </c>
       <c r="B6" t="n">
-        <v>0.82</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9213483146067416</v>
+        <v>0.9222222222222223</v>
       </c>
       <c r="D6" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8137254901960784</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8586387434554974</v>
+        <v>0.8645833333333334</v>
       </c>
       <c r="F6" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G6" t="n">
         <v>41</v>
@@ -710,7 +710,7 @@
         <v>7</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -833,25 +833,25 @@
         <v>0.7666666666666667</v>
       </c>
       <c r="C9" t="n">
-        <v>0.935064935064935</v>
+        <v>0.9135802469135802</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7254901960784313</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8044692737430168</v>
+        <v>0.8087431693989071</v>
       </c>
       <c r="F9" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G9" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -880,25 +880,25 @@
         <v>0.7466666666666667</v>
       </c>
       <c r="C10" t="n">
-        <v>0.75</v>
+        <v>0.7424242424242424</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9607843137254902</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8347826086956521</v>
+        <v>0.8376068376068376</v>
       </c>
       <c r="F10" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1253,19 +1253,19 @@
         <v>150</v>
       </c>
       <c r="B18" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8695652173913043</v>
+        <v>0.875</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.823529411764706</v>
       </c>
       <c r="F18" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G18" t="n">
         <v>120</v>
@@ -1274,7 +1274,7 @@
         <v>3</v>
       </c>
       <c r="I18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1303,25 +1303,25 @@
         <v>0.7466666666666667</v>
       </c>
       <c r="C19" t="n">
-        <v>0.4098360655737705</v>
+        <v>0.4126984126984127</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9629629629629629</v>
       </c>
       <c r="E19" t="n">
-        <v>0.5681818181818182</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G19" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1488,25 +1488,25 @@
         <v>150</v>
       </c>
       <c r="B23" t="n">
-        <v>0.88</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="D23" t="n">
         <v>0.9523809523809523</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6896551724137931</v>
+        <v>0.6779661016949152</v>
       </c>
       <c r="F23" t="n">
         <v>20</v>
       </c>
       <c r="G23" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -1676,25 +1676,25 @@
         <v>150</v>
       </c>
       <c r="B27" t="n">
-        <v>0.86</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5</v>
+        <v>0.4838709677419355</v>
       </c>
       <c r="D27" t="n">
         <v>0.7142857142857143</v>
       </c>
       <c r="E27" t="n">
-        <v>0.588235294117647</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="F27" t="n">
         <v>15</v>
       </c>
       <c r="G27" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I27" t="n">
         <v>6</v>
@@ -1723,25 +1723,25 @@
         <v>150</v>
       </c>
       <c r="B28" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="C28" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4222222222222222</v>
       </c>
       <c r="D28" t="n">
         <v>0.9047619047619048</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6031746031746031</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="F28" t="n">
         <v>19</v>
       </c>
       <c r="G28" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H28" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I28" t="n">
         <v>2</v>
@@ -1770,25 +1770,25 @@
         <v>150</v>
       </c>
       <c r="B29" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="C29" t="n">
-        <v>0.625</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="D29" t="n">
         <v>0.6818181818181818</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6521739130434783</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F29" t="n">
         <v>15</v>
       </c>
       <c r="G29" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H29" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I29" t="n">
         <v>7</v>
@@ -2193,25 +2193,25 @@
         <v>150</v>
       </c>
       <c r="B38" t="n">
-        <v>0.7</v>
+        <v>0.7066666666666667</v>
       </c>
       <c r="C38" t="n">
-        <v>0.8591549295774648</v>
+        <v>0.8714285714285714</v>
       </c>
       <c r="D38" t="n">
         <v>0.6354166666666666</v>
       </c>
       <c r="E38" t="n">
-        <v>0.7305389221556885</v>
+        <v>0.7349397590361446</v>
       </c>
       <c r="F38" t="n">
         <v>61</v>
       </c>
       <c r="G38" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I38" t="n">
         <v>35</v>
@@ -2240,25 +2240,25 @@
         <v>150</v>
       </c>
       <c r="B39" t="n">
-        <v>0.72</v>
+        <v>0.7266666666666667</v>
       </c>
       <c r="C39" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.8767123287671232</v>
       </c>
       <c r="D39" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="E39" t="n">
-        <v>0.7529411764705882</v>
+        <v>0.7573964497041421</v>
       </c>
       <c r="F39" t="n">
         <v>64</v>
       </c>
       <c r="G39" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I39" t="n">
         <v>32</v>
@@ -2334,25 +2334,25 @@
         <v>150</v>
       </c>
       <c r="B41" t="n">
-        <v>0.7066666666666667</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="C41" t="n">
-        <v>0.8939393939393939</v>
+        <v>0.855072463768116</v>
       </c>
       <c r="D41" t="n">
         <v>0.6145833333333334</v>
       </c>
       <c r="E41" t="n">
-        <v>0.7283950617283952</v>
+        <v>0.7151515151515152</v>
       </c>
       <c r="F41" t="n">
         <v>59</v>
       </c>
       <c r="G41" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H41" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I41" t="n">
         <v>37</v>
@@ -2522,25 +2522,25 @@
         <v>150</v>
       </c>
       <c r="B45" t="n">
-        <v>0.6933333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="C45" t="n">
-        <v>0.9464285714285714</v>
+        <v>0.9137931034482759</v>
       </c>
       <c r="D45" t="n">
         <v>0.5520833333333334</v>
       </c>
       <c r="E45" t="n">
-        <v>0.6973684210526316</v>
+        <v>0.6883116883116883</v>
       </c>
       <c r="F45" t="n">
         <v>53</v>
       </c>
       <c r="G45" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
         <v>43</v>
@@ -2569,25 +2569,25 @@
         <v>150</v>
       </c>
       <c r="B46" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C46" t="n">
-        <v>0.8051948051948052</v>
+        <v>0.7948717948717948</v>
       </c>
       <c r="D46" t="n">
         <v>0.6458333333333334</v>
       </c>
       <c r="E46" t="n">
-        <v>0.7167630057803468</v>
+        <v>0.7126436781609194</v>
       </c>
       <c r="F46" t="n">
         <v>62</v>
       </c>
       <c r="G46" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H46" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I46" t="n">
         <v>34</v>
@@ -2616,25 +2616,25 @@
         <v>150</v>
       </c>
       <c r="B47" t="n">
-        <v>0.6333333333333333</v>
+        <v>0.6266666666666667</v>
       </c>
       <c r="C47" t="n">
-        <v>0.9347826086956522</v>
+        <v>0.9148936170212766</v>
       </c>
       <c r="D47" t="n">
         <v>0.4526315789473684</v>
       </c>
       <c r="E47" t="n">
-        <v>0.6099290780141844</v>
+        <v>0.6056338028169014</v>
       </c>
       <c r="F47" t="n">
         <v>43</v>
       </c>
       <c r="G47" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I47" t="n">
         <v>52</v>
@@ -2663,25 +2663,25 @@
         <v>150</v>
       </c>
       <c r="B48" t="n">
-        <v>0.7466666666666667</v>
+        <v>0.7533333333333333</v>
       </c>
       <c r="C48" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.9264705882352942</v>
       </c>
       <c r="D48" t="n">
         <v>0.6631578947368421</v>
       </c>
       <c r="E48" t="n">
-        <v>0.7682926829268292</v>
+        <v>0.773006134969325</v>
       </c>
       <c r="F48" t="n">
         <v>63</v>
       </c>
       <c r="G48" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I48" t="n">
         <v>32</v>
@@ -2992,25 +2992,25 @@
         <v>150</v>
       </c>
       <c r="B55" t="n">
-        <v>0.6266666666666667</v>
+        <v>0.62</v>
       </c>
       <c r="C55" t="n">
-        <v>0.8</v>
+        <v>0.7878787878787878</v>
       </c>
       <c r="D55" t="n">
         <v>0.5473684210526316</v>
       </c>
       <c r="E55" t="n">
-        <v>0.65</v>
+        <v>0.6459627329192547</v>
       </c>
       <c r="F55" t="n">
         <v>52</v>
       </c>
       <c r="G55" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H55" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I55" t="n">
         <v>43</v>
@@ -3086,25 +3086,25 @@
         <v>150</v>
       </c>
       <c r="B57" t="n">
-        <v>0.7666666666666667</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C57" t="n">
-        <v>0.8939393939393939</v>
+        <v>0.9076923076923077</v>
       </c>
       <c r="D57" t="n">
         <v>0.6781609195402298</v>
       </c>
       <c r="E57" t="n">
-        <v>0.7712418300653594</v>
+        <v>0.7763157894736842</v>
       </c>
       <c r="F57" t="n">
         <v>59</v>
       </c>
       <c r="G57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I57" t="n">
         <v>28</v>
@@ -3462,28 +3462,28 @@
         <v>150</v>
       </c>
       <c r="B65" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.9533333333333334</v>
       </c>
       <c r="C65" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D65" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E65" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="F65" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" t="n">
+        <v>139</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2</v>
+      </c>
+      <c r="I65" t="n">
         <v>5</v>
-      </c>
-      <c r="G65" t="n">
-        <v>140</v>
-      </c>
-      <c r="H65" t="n">
-        <v>1</v>
-      </c>
-      <c r="I65" t="n">
-        <v>4</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -3509,19 +3509,19 @@
         <v>150</v>
       </c>
       <c r="B66" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.96</v>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E66" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.5</v>
       </c>
       <c r="F66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66" t="n">
         <v>141</v>
@@ -3530,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -3791,19 +3791,19 @@
         <v>150</v>
       </c>
       <c r="B72" t="n">
-        <v>0.9266666666666666</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="C72" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="D72" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E72" t="n">
-        <v>0.1538461538461538</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" t="n">
         <v>138</v>
@@ -3812,7 +3812,7 @@
         <v>3</v>
       </c>
       <c r="I72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -3838,19 +3838,19 @@
         <v>150</v>
       </c>
       <c r="B73" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.82</v>
       </c>
       <c r="C73" t="n">
-        <v>0.12</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="D73" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E73" t="n">
-        <v>0.1764705882352941</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G73" t="n">
         <v>119</v>
@@ -3859,7 +3859,7 @@
         <v>22</v>
       </c>
       <c r="I73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -3885,25 +3885,25 @@
         <v>150</v>
       </c>
       <c r="B74" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5266666666666666</v>
       </c>
       <c r="C74" t="n">
-        <v>0.72</v>
+        <v>0.7105263157894737</v>
       </c>
       <c r="D74" t="n">
         <v>0.5242718446601942</v>
       </c>
       <c r="E74" t="n">
-        <v>0.6067415730337079</v>
+        <v>0.6033519553072626</v>
       </c>
       <c r="F74" t="n">
         <v>54</v>
       </c>
       <c r="G74" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H74" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I74" t="n">
         <v>49</v>
@@ -3932,25 +3932,25 @@
         <v>150</v>
       </c>
       <c r="B75" t="n">
-        <v>0.6066666666666667</v>
+        <v>0.6133333333333333</v>
       </c>
       <c r="C75" t="n">
-        <v>0.7340425531914894</v>
+        <v>0.7419354838709677</v>
       </c>
       <c r="D75" t="n">
         <v>0.6699029126213593</v>
       </c>
       <c r="E75" t="n">
-        <v>0.7005076142131981</v>
+        <v>0.7040816326530613</v>
       </c>
       <c r="F75" t="n">
         <v>69</v>
       </c>
       <c r="G75" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H75" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I75" t="n">
         <v>34</v>
@@ -4073,25 +4073,25 @@
         <v>150</v>
       </c>
       <c r="B78" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6533333333333333</v>
       </c>
       <c r="C78" t="n">
-        <v>0.8271604938271605</v>
+        <v>0.8072289156626506</v>
       </c>
       <c r="D78" t="n">
         <v>0.6504854368932039</v>
       </c>
       <c r="E78" t="n">
-        <v>0.7282608695652175</v>
+        <v>0.7204301075268817</v>
       </c>
       <c r="F78" t="n">
         <v>67</v>
       </c>
       <c r="G78" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H78" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I78" t="n">
         <v>36</v>
@@ -4214,25 +4214,25 @@
         <v>150</v>
       </c>
       <c r="B81" t="n">
-        <v>0.5466666666666666</v>
+        <v>0.5533333333333333</v>
       </c>
       <c r="C81" t="n">
-        <v>0.7868852459016393</v>
+        <v>0.8</v>
       </c>
       <c r="D81" t="n">
         <v>0.4660194174757282</v>
       </c>
       <c r="E81" t="n">
-        <v>0.5853658536585367</v>
+        <v>0.588957055214724</v>
       </c>
       <c r="F81" t="n">
         <v>48</v>
       </c>
       <c r="G81" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H81" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I81" t="n">
         <v>55</v>
@@ -4261,25 +4261,25 @@
         <v>150</v>
       </c>
       <c r="B82" t="n">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="C82" t="n">
-        <v>0.801980198019802</v>
+        <v>0.7788461538461539</v>
       </c>
       <c r="D82" t="n">
         <v>0.7864077669902912</v>
       </c>
       <c r="E82" t="n">
-        <v>0.7941176470588236</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="F82" t="n">
         <v>81</v>
       </c>
       <c r="G82" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H82" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I82" t="n">
         <v>22</v>
@@ -4355,25 +4355,25 @@
         <v>150</v>
       </c>
       <c r="B84" t="n">
-        <v>0.7666666666666667</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="C84" t="n">
-        <v>0.8387096774193549</v>
+        <v>0.8813559322033898</v>
       </c>
       <c r="D84" t="n">
         <v>0.6753246753246753</v>
       </c>
       <c r="E84" t="n">
-        <v>0.7482014388489209</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="F84" t="n">
         <v>52</v>
       </c>
       <c r="G84" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H84" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I84" t="n">
         <v>25</v>
@@ -4496,25 +4496,25 @@
         <v>150</v>
       </c>
       <c r="B87" t="n">
-        <v>0.7466666666666667</v>
+        <v>0.74</v>
       </c>
       <c r="C87" t="n">
-        <v>0.8979591836734694</v>
+        <v>0.88</v>
       </c>
       <c r="D87" t="n">
         <v>0.5714285714285714</v>
       </c>
       <c r="E87" t="n">
-        <v>0.6984126984126985</v>
+        <v>0.6929133858267715</v>
       </c>
       <c r="F87" t="n">
         <v>44</v>
       </c>
       <c r="G87" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H87" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I87" t="n">
         <v>33</v>
@@ -4684,25 +4684,25 @@
         <v>150</v>
       </c>
       <c r="B91" t="n">
-        <v>0.72</v>
+        <v>0.7066666666666667</v>
       </c>
       <c r="C91" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8113207547169812</v>
       </c>
       <c r="D91" t="n">
         <v>0.5584415584415584</v>
       </c>
       <c r="E91" t="n">
-        <v>0.671875</v>
+        <v>0.6615384615384615</v>
       </c>
       <c r="F91" t="n">
         <v>43</v>
       </c>
       <c r="G91" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H91" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I91" t="n">
         <v>34</v>
@@ -4778,19 +4778,19 @@
         <v>150</v>
       </c>
       <c r="B93" t="n">
-        <v>0.7133333333333334</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="C93" t="n">
-        <v>0.9516129032258065</v>
+        <v>0.9538461538461539</v>
       </c>
       <c r="D93" t="n">
-        <v>0.5959595959595959</v>
+        <v>0.6262626262626263</v>
       </c>
       <c r="E93" t="n">
-        <v>0.732919254658385</v>
+        <v>0.7560975609756098</v>
       </c>
       <c r="F93" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G93" t="n">
         <v>48</v>
@@ -4799,7 +4799,7 @@
         <v>3</v>
       </c>
       <c r="I93" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5154,25 +5154,25 @@
         <v>150</v>
       </c>
       <c r="B101" t="n">
-        <v>0.78</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="C101" t="n">
-        <v>0.5957446808510638</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="D101" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="E101" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.6363636363636365</v>
       </c>
       <c r="F101" t="n">
         <v>28</v>
       </c>
       <c r="G101" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H101" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I101" t="n">
         <v>14</v>
@@ -5201,25 +5201,25 @@
         <v>150</v>
       </c>
       <c r="B102" t="n">
-        <v>0.82</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C102" t="n">
-        <v>0.6229508196721312</v>
+        <v>0.6440677966101694</v>
       </c>
       <c r="D102" t="n">
         <v>0.9047619047619048</v>
       </c>
       <c r="E102" t="n">
-        <v>0.7378640776699029</v>
+        <v>0.7524752475247525</v>
       </c>
       <c r="F102" t="n">
         <v>38</v>
       </c>
       <c r="G102" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H102" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I102" t="n">
         <v>4</v>
@@ -5483,25 +5483,25 @@
         <v>150</v>
       </c>
       <c r="B108" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="C108" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D108" t="n">
         <v>0.6190476190476191</v>
       </c>
       <c r="E108" t="n">
-        <v>0.6500000000000001</v>
+        <v>0.6419753086419754</v>
       </c>
       <c r="F108" t="n">
         <v>26</v>
       </c>
       <c r="G108" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H108" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I108" t="n">
         <v>16</v>
@@ -5530,25 +5530,25 @@
         <v>150</v>
       </c>
       <c r="B109" t="n">
-        <v>0.7066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="C109" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="D109" t="n">
         <v>0.8571428571428571</v>
       </c>
       <c r="E109" t="n">
-        <v>0.6206896551724138</v>
+        <v>0.6</v>
       </c>
       <c r="F109" t="n">
         <v>36</v>
       </c>
       <c r="G109" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H109" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I109" t="n">
         <v>6</v>
@@ -5765,25 +5765,25 @@
         <v>150</v>
       </c>
       <c r="B114" t="n">
-        <v>0.9466666666666667</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C114" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.6842105263157895</v>
       </c>
       <c r="D114" t="n">
         <v>0.8125</v>
       </c>
       <c r="E114" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.742857142857143</v>
       </c>
       <c r="F114" t="n">
         <v>13</v>
       </c>
       <c r="G114" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I114" t="n">
         <v>3</v>
@@ -5953,25 +5953,25 @@
         <v>150</v>
       </c>
       <c r="B118" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.9</v>
       </c>
       <c r="C118" t="n">
-        <v>0.5357142857142857</v>
+        <v>0.5172413793103449</v>
       </c>
       <c r="D118" t="n">
         <v>0.9375</v>
       </c>
       <c r="E118" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="F118" t="n">
         <v>15</v>
       </c>
       <c r="G118" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H118" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I118" t="n">
         <v>1</v>
@@ -6000,25 +6000,25 @@
         <v>150</v>
       </c>
       <c r="B119" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.7933333333333333</v>
       </c>
       <c r="C119" t="n">
-        <v>0.7068965517241379</v>
+        <v>0.7454545454545455</v>
       </c>
       <c r="D119" t="n">
         <v>0.7068965517241379</v>
       </c>
       <c r="E119" t="n">
-        <v>0.7068965517241379</v>
+        <v>0.7256637168141592</v>
       </c>
       <c r="F119" t="n">
         <v>41</v>
       </c>
       <c r="G119" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H119" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I119" t="n">
         <v>17</v>
@@ -6050,25 +6050,25 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C120" t="n">
-        <v>0.72</v>
+        <v>0.726027397260274</v>
       </c>
       <c r="D120" t="n">
-        <v>0.9310344827586207</v>
+        <v>0.9137931034482759</v>
       </c>
       <c r="E120" t="n">
-        <v>0.8120300751879699</v>
+        <v>0.8091603053435115</v>
       </c>
       <c r="F120" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G120" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H120" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I120" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -6329,25 +6329,25 @@
         <v>150</v>
       </c>
       <c r="B126" t="n">
-        <v>0.7866666666666666</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C126" t="n">
-        <v>0.75</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="D126" t="n">
         <v>0.6724137931034483</v>
       </c>
       <c r="E126" t="n">
-        <v>0.709090909090909</v>
+        <v>0.6964285714285714</v>
       </c>
       <c r="F126" t="n">
         <v>39</v>
       </c>
       <c r="G126" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H126" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I126" t="n">
         <v>19</v>
@@ -6376,28 +6376,28 @@
         <v>150</v>
       </c>
       <c r="B127" t="n">
-        <v>0.62</v>
+        <v>0.6066666666666667</v>
       </c>
       <c r="C127" t="n">
-        <v>0.504950495049505</v>
+        <v>0.4952380952380953</v>
       </c>
       <c r="D127" t="n">
-        <v>0.8793103448275862</v>
+        <v>0.896551724137931</v>
       </c>
       <c r="E127" t="n">
-        <v>0.6415094339622641</v>
+        <v>0.6380368098159509</v>
       </c>
       <c r="F127" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G127" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H127" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I127" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -6470,25 +6470,25 @@
         <v>150</v>
       </c>
       <c r="B129" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.7133333333333334</v>
       </c>
       <c r="C129" t="n">
-        <v>0.7547169811320755</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D129" t="n">
         <v>0.5970149253731343</v>
       </c>
       <c r="E129" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6504065040650405</v>
       </c>
       <c r="F129" t="n">
         <v>40</v>
       </c>
       <c r="G129" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H129" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I129" t="n">
         <v>27</v>
@@ -6564,25 +6564,25 @@
         <v>150</v>
       </c>
       <c r="B131" t="n">
-        <v>0.4066666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="C131" t="n">
-        <v>0.392156862745098</v>
+        <v>0.3883495145631068</v>
       </c>
       <c r="D131" t="n">
         <v>0.5970149253731343</v>
       </c>
       <c r="E131" t="n">
-        <v>0.4733727810650887</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="F131" t="n">
         <v>40</v>
       </c>
       <c r="G131" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H131" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I131" t="n">
         <v>27</v>
@@ -6611,25 +6611,25 @@
         <v>150</v>
       </c>
       <c r="B132" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.62</v>
       </c>
       <c r="C132" t="n">
-        <v>0.84</v>
+        <v>0.65625</v>
       </c>
       <c r="D132" t="n">
         <v>0.3134328358208955</v>
       </c>
       <c r="E132" t="n">
-        <v>0.4565217391304348</v>
+        <v>0.4242424242424243</v>
       </c>
       <c r="F132" t="n">
         <v>21</v>
       </c>
       <c r="G132" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="H132" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I132" t="n">
         <v>46</v>
@@ -6799,25 +6799,25 @@
         <v>150</v>
       </c>
       <c r="B136" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5266666666666666</v>
       </c>
       <c r="C136" t="n">
-        <v>0.4805194805194805</v>
+        <v>0.4743589743589743</v>
       </c>
       <c r="D136" t="n">
         <v>0.5522388059701493</v>
       </c>
       <c r="E136" t="n">
-        <v>0.5138888888888888</v>
+        <v>0.5103448275862068</v>
       </c>
       <c r="F136" t="n">
         <v>37</v>
       </c>
       <c r="G136" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H136" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I136" t="n">
         <v>30</v>
@@ -6849,25 +6849,25 @@
         <v>0.6066666666666667</v>
       </c>
       <c r="C137" t="n">
-        <v>0.5102040816326531</v>
+        <v>0.5098039215686274</v>
       </c>
       <c r="D137" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="E137" t="n">
-        <v>0.4587155963302753</v>
+        <v>0.4684684684684685</v>
       </c>
       <c r="F137" t="n">
+        <v>26</v>
+      </c>
+      <c r="G137" t="n">
+        <v>65</v>
+      </c>
+      <c r="H137" t="n">
         <v>25</v>
       </c>
-      <c r="G137" t="n">
-        <v>66</v>
-      </c>
-      <c r="H137" t="n">
-        <v>24</v>
-      </c>
       <c r="I137" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
@@ -6893,25 +6893,25 @@
         <v>150</v>
       </c>
       <c r="B138" t="n">
-        <v>0.7533333333333333</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="C138" t="n">
-        <v>0.7346938775510204</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="D138" t="n">
         <v>0.6</v>
       </c>
       <c r="E138" t="n">
-        <v>0.6605504587155964</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F138" t="n">
         <v>36</v>
       </c>
       <c r="G138" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H138" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I138" t="n">
         <v>24</v>
@@ -6987,25 +6987,25 @@
         <v>150</v>
       </c>
       <c r="B140" t="n">
-        <v>0.3466666666666667</v>
+        <v>0.34</v>
       </c>
       <c r="C140" t="n">
-        <v>0.2934782608695652</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="D140" t="n">
         <v>0.45</v>
       </c>
       <c r="E140" t="n">
-        <v>0.3552631578947368</v>
+        <v>0.3529411764705882</v>
       </c>
       <c r="F140" t="n">
         <v>27</v>
       </c>
       <c r="G140" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H140" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I140" t="n">
         <v>33</v>
@@ -7225,25 +7225,25 @@
         <v>0.52</v>
       </c>
       <c r="C145" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D145" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.35</v>
       </c>
       <c r="E145" t="n">
-        <v>0.3571428571428571</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="F145" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G145" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H145" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I145" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J145" t="inlineStr">
         <is>
@@ -7350,25 +7350,25 @@
         <v>150</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.86</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9263157894736842</v>
       </c>
       <c r="D2" t="n">
         <v>0.8627450980392157</v>
       </c>
       <c r="E2" t="n">
-        <v>0.888888888888889</v>
+        <v>0.8934010152284264</v>
       </c>
       <c r="F2" t="n">
         <v>88</v>
       </c>
       <c r="G2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2" t="n">
         <v>14</v>
@@ -7397,19 +7397,19 @@
         <v>150</v>
       </c>
       <c r="B3" t="n">
-        <v>0.92</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9215686274509803</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9306930693069307</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G3" t="n">
         <v>42</v>
@@ -7418,7 +7418,7 @@
         <v>6</v>
       </c>
       <c r="I3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -7491,19 +7491,19 @@
         <v>150</v>
       </c>
       <c r="B5" t="n">
-        <v>0.76</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9125</v>
+        <v>0.9146341463414634</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7156862745098039</v>
+        <v>0.7352941176470589</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8021978021978022</v>
+        <v>0.8152173913043479</v>
       </c>
       <c r="F5" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
         <v>41</v>
@@ -7512,7 +7512,7 @@
         <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -7538,19 +7538,19 @@
         <v>150</v>
       </c>
       <c r="B6" t="n">
-        <v>0.82</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9213483146067416</v>
+        <v>0.9222222222222223</v>
       </c>
       <c r="D6" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8137254901960784</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8586387434554974</v>
+        <v>0.8645833333333334</v>
       </c>
       <c r="F6" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G6" t="n">
         <v>41</v>
@@ -7559,7 +7559,7 @@
         <v>7</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -7682,25 +7682,25 @@
         <v>0.7666666666666667</v>
       </c>
       <c r="C9" t="n">
-        <v>0.935064935064935</v>
+        <v>0.9135802469135802</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7254901960784313</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8044692737430168</v>
+        <v>0.8087431693989071</v>
       </c>
       <c r="F9" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G9" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -7729,25 +7729,25 @@
         <v>0.7466666666666667</v>
       </c>
       <c r="C10" t="n">
-        <v>0.75</v>
+        <v>0.7424242424242424</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9607843137254902</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8347826086956521</v>
+        <v>0.8376068376068376</v>
       </c>
       <c r="F10" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -8102,19 +8102,19 @@
         <v>150</v>
       </c>
       <c r="B18" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8695652173913043</v>
+        <v>0.875</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.823529411764706</v>
       </c>
       <c r="F18" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G18" t="n">
         <v>120</v>
@@ -8123,7 +8123,7 @@
         <v>3</v>
       </c>
       <c r="I18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -8152,25 +8152,25 @@
         <v>0.7466666666666667</v>
       </c>
       <c r="C19" t="n">
-        <v>0.4098360655737705</v>
+        <v>0.4126984126984127</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9629629629629629</v>
       </c>
       <c r="E19" t="n">
-        <v>0.5681818181818182</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G19" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -8337,25 +8337,25 @@
         <v>150</v>
       </c>
       <c r="B23" t="n">
-        <v>0.88</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="D23" t="n">
         <v>0.9523809523809523</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6896551724137931</v>
+        <v>0.6779661016949152</v>
       </c>
       <c r="F23" t="n">
         <v>20</v>
       </c>
       <c r="G23" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -8525,25 +8525,25 @@
         <v>150</v>
       </c>
       <c r="B27" t="n">
-        <v>0.86</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5</v>
+        <v>0.4838709677419355</v>
       </c>
       <c r="D27" t="n">
         <v>0.7142857142857143</v>
       </c>
       <c r="E27" t="n">
-        <v>0.588235294117647</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="F27" t="n">
         <v>15</v>
       </c>
       <c r="G27" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I27" t="n">
         <v>6</v>
@@ -8572,25 +8572,25 @@
         <v>150</v>
       </c>
       <c r="B28" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="C28" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4222222222222222</v>
       </c>
       <c r="D28" t="n">
         <v>0.9047619047619048</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6031746031746031</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="F28" t="n">
         <v>19</v>
       </c>
       <c r="G28" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H28" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I28" t="n">
         <v>2</v>
@@ -8619,25 +8619,25 @@
         <v>150</v>
       </c>
       <c r="B29" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="C29" t="n">
-        <v>0.625</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="D29" t="n">
         <v>0.6818181818181818</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6521739130434783</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F29" t="n">
         <v>15</v>
       </c>
       <c r="G29" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H29" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I29" t="n">
         <v>7</v>
@@ -9042,25 +9042,25 @@
         <v>150</v>
       </c>
       <c r="B38" t="n">
-        <v>0.7</v>
+        <v>0.7066666666666667</v>
       </c>
       <c r="C38" t="n">
-        <v>0.8591549295774648</v>
+        <v>0.8714285714285714</v>
       </c>
       <c r="D38" t="n">
         <v>0.6354166666666666</v>
       </c>
       <c r="E38" t="n">
-        <v>0.7305389221556885</v>
+        <v>0.7349397590361446</v>
       </c>
       <c r="F38" t="n">
         <v>61</v>
       </c>
       <c r="G38" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I38" t="n">
         <v>35</v>
@@ -9089,25 +9089,25 @@
         <v>150</v>
       </c>
       <c r="B39" t="n">
-        <v>0.72</v>
+        <v>0.7266666666666667</v>
       </c>
       <c r="C39" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.8767123287671232</v>
       </c>
       <c r="D39" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="E39" t="n">
-        <v>0.7529411764705882</v>
+        <v>0.7573964497041421</v>
       </c>
       <c r="F39" t="n">
         <v>64</v>
       </c>
       <c r="G39" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I39" t="n">
         <v>32</v>
@@ -9183,25 +9183,25 @@
         <v>150</v>
       </c>
       <c r="B41" t="n">
-        <v>0.7066666666666667</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="C41" t="n">
-        <v>0.8939393939393939</v>
+        <v>0.855072463768116</v>
       </c>
       <c r="D41" t="n">
         <v>0.6145833333333334</v>
       </c>
       <c r="E41" t="n">
-        <v>0.7283950617283952</v>
+        <v>0.7151515151515152</v>
       </c>
       <c r="F41" t="n">
         <v>59</v>
       </c>
       <c r="G41" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H41" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I41" t="n">
         <v>37</v>
@@ -9371,25 +9371,25 @@
         <v>150</v>
       </c>
       <c r="B45" t="n">
-        <v>0.6933333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="C45" t="n">
-        <v>0.9464285714285714</v>
+        <v>0.9137931034482759</v>
       </c>
       <c r="D45" t="n">
         <v>0.5520833333333334</v>
       </c>
       <c r="E45" t="n">
-        <v>0.6973684210526316</v>
+        <v>0.6883116883116883</v>
       </c>
       <c r="F45" t="n">
         <v>53</v>
       </c>
       <c r="G45" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
         <v>43</v>
@@ -9418,25 +9418,25 @@
         <v>150</v>
       </c>
       <c r="B46" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C46" t="n">
-        <v>0.8051948051948052</v>
+        <v>0.7948717948717948</v>
       </c>
       <c r="D46" t="n">
         <v>0.6458333333333334</v>
       </c>
       <c r="E46" t="n">
-        <v>0.7167630057803468</v>
+        <v>0.7126436781609194</v>
       </c>
       <c r="F46" t="n">
         <v>62</v>
       </c>
       <c r="G46" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H46" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I46" t="n">
         <v>34</v>
@@ -9465,25 +9465,25 @@
         <v>150</v>
       </c>
       <c r="B47" t="n">
-        <v>0.6333333333333333</v>
+        <v>0.6266666666666667</v>
       </c>
       <c r="C47" t="n">
-        <v>0.9347826086956522</v>
+        <v>0.9148936170212766</v>
       </c>
       <c r="D47" t="n">
         <v>0.4526315789473684</v>
       </c>
       <c r="E47" t="n">
-        <v>0.6099290780141844</v>
+        <v>0.6056338028169014</v>
       </c>
       <c r="F47" t="n">
         <v>43</v>
       </c>
       <c r="G47" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I47" t="n">
         <v>52</v>
@@ -9512,25 +9512,25 @@
         <v>150</v>
       </c>
       <c r="B48" t="n">
-        <v>0.7466666666666667</v>
+        <v>0.7533333333333333</v>
       </c>
       <c r="C48" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.9264705882352942</v>
       </c>
       <c r="D48" t="n">
         <v>0.6631578947368421</v>
       </c>
       <c r="E48" t="n">
-        <v>0.7682926829268292</v>
+        <v>0.773006134969325</v>
       </c>
       <c r="F48" t="n">
         <v>63</v>
       </c>
       <c r="G48" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I48" t="n">
         <v>32</v>
@@ -9841,25 +9841,25 @@
         <v>150</v>
       </c>
       <c r="B55" t="n">
-        <v>0.6266666666666667</v>
+        <v>0.62</v>
       </c>
       <c r="C55" t="n">
-        <v>0.8</v>
+        <v>0.7878787878787878</v>
       </c>
       <c r="D55" t="n">
         <v>0.5473684210526316</v>
       </c>
       <c r="E55" t="n">
-        <v>0.65</v>
+        <v>0.6459627329192547</v>
       </c>
       <c r="F55" t="n">
         <v>52</v>
       </c>
       <c r="G55" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H55" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I55" t="n">
         <v>43</v>
@@ -9935,25 +9935,25 @@
         <v>150</v>
       </c>
       <c r="B57" t="n">
-        <v>0.7666666666666667</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C57" t="n">
-        <v>0.8939393939393939</v>
+        <v>0.9076923076923077</v>
       </c>
       <c r="D57" t="n">
         <v>0.6781609195402298</v>
       </c>
       <c r="E57" t="n">
-        <v>0.7712418300653594</v>
+        <v>0.7763157894736842</v>
       </c>
       <c r="F57" t="n">
         <v>59</v>
       </c>
       <c r="G57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I57" t="n">
         <v>28</v>
@@ -10311,28 +10311,28 @@
         <v>150</v>
       </c>
       <c r="B65" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.9533333333333334</v>
       </c>
       <c r="C65" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D65" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E65" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="F65" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" t="n">
+        <v>139</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2</v>
+      </c>
+      <c r="I65" t="n">
         <v>5</v>
-      </c>
-      <c r="G65" t="n">
-        <v>140</v>
-      </c>
-      <c r="H65" t="n">
-        <v>1</v>
-      </c>
-      <c r="I65" t="n">
-        <v>4</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -10358,19 +10358,19 @@
         <v>150</v>
       </c>
       <c r="B66" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.96</v>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E66" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.5</v>
       </c>
       <c r="F66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66" t="n">
         <v>141</v>
@@ -10379,7 +10379,7 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -10640,19 +10640,19 @@
         <v>150</v>
       </c>
       <c r="B72" t="n">
-        <v>0.9266666666666666</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="C72" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="D72" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E72" t="n">
-        <v>0.1538461538461538</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" t="n">
         <v>138</v>
@@ -10661,7 +10661,7 @@
         <v>3</v>
       </c>
       <c r="I72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -10687,19 +10687,19 @@
         <v>150</v>
       </c>
       <c r="B73" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.82</v>
       </c>
       <c r="C73" t="n">
-        <v>0.12</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="D73" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E73" t="n">
-        <v>0.1764705882352941</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G73" t="n">
         <v>119</v>
@@ -10708,7 +10708,7 @@
         <v>22</v>
       </c>
       <c r="I73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -10734,25 +10734,25 @@
         <v>150</v>
       </c>
       <c r="B74" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5266666666666666</v>
       </c>
       <c r="C74" t="n">
-        <v>0.72</v>
+        <v>0.7105263157894737</v>
       </c>
       <c r="D74" t="n">
         <v>0.5242718446601942</v>
       </c>
       <c r="E74" t="n">
-        <v>0.6067415730337079</v>
+        <v>0.6033519553072626</v>
       </c>
       <c r="F74" t="n">
         <v>54</v>
       </c>
       <c r="G74" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H74" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I74" t="n">
         <v>49</v>
@@ -10781,25 +10781,25 @@
         <v>150</v>
       </c>
       <c r="B75" t="n">
-        <v>0.6066666666666667</v>
+        <v>0.6133333333333333</v>
       </c>
       <c r="C75" t="n">
-        <v>0.7340425531914894</v>
+        <v>0.7419354838709677</v>
       </c>
       <c r="D75" t="n">
         <v>0.6699029126213593</v>
       </c>
       <c r="E75" t="n">
-        <v>0.7005076142131981</v>
+        <v>0.7040816326530613</v>
       </c>
       <c r="F75" t="n">
         <v>69</v>
       </c>
       <c r="G75" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H75" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I75" t="n">
         <v>34</v>
@@ -10922,25 +10922,25 @@
         <v>150</v>
       </c>
       <c r="B78" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6533333333333333</v>
       </c>
       <c r="C78" t="n">
-        <v>0.8271604938271605</v>
+        <v>0.8072289156626506</v>
       </c>
       <c r="D78" t="n">
         <v>0.6504854368932039</v>
       </c>
       <c r="E78" t="n">
-        <v>0.7282608695652175</v>
+        <v>0.7204301075268817</v>
       </c>
       <c r="F78" t="n">
         <v>67</v>
       </c>
       <c r="G78" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H78" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I78" t="n">
         <v>36</v>
@@ -11063,25 +11063,25 @@
         <v>150</v>
       </c>
       <c r="B81" t="n">
-        <v>0.5466666666666666</v>
+        <v>0.5533333333333333</v>
       </c>
       <c r="C81" t="n">
-        <v>0.7868852459016393</v>
+        <v>0.8</v>
       </c>
       <c r="D81" t="n">
         <v>0.4660194174757282</v>
       </c>
       <c r="E81" t="n">
-        <v>0.5853658536585367</v>
+        <v>0.588957055214724</v>
       </c>
       <c r="F81" t="n">
         <v>48</v>
       </c>
       <c r="G81" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H81" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I81" t="n">
         <v>55</v>
@@ -11110,25 +11110,25 @@
         <v>150</v>
       </c>
       <c r="B82" t="n">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="C82" t="n">
-        <v>0.801980198019802</v>
+        <v>0.7788461538461539</v>
       </c>
       <c r="D82" t="n">
         <v>0.7864077669902912</v>
       </c>
       <c r="E82" t="n">
-        <v>0.7941176470588236</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="F82" t="n">
         <v>81</v>
       </c>
       <c r="G82" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H82" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I82" t="n">
         <v>22</v>
@@ -11204,25 +11204,25 @@
         <v>150</v>
       </c>
       <c r="B84" t="n">
-        <v>0.7666666666666667</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="C84" t="n">
-        <v>0.8387096774193549</v>
+        <v>0.8813559322033898</v>
       </c>
       <c r="D84" t="n">
         <v>0.6753246753246753</v>
       </c>
       <c r="E84" t="n">
-        <v>0.7482014388489209</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="F84" t="n">
         <v>52</v>
       </c>
       <c r="G84" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H84" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I84" t="n">
         <v>25</v>
@@ -11345,25 +11345,25 @@
         <v>150</v>
       </c>
       <c r="B87" t="n">
-        <v>0.7466666666666667</v>
+        <v>0.74</v>
       </c>
       <c r="C87" t="n">
-        <v>0.8979591836734694</v>
+        <v>0.88</v>
       </c>
       <c r="D87" t="n">
         <v>0.5714285714285714</v>
       </c>
       <c r="E87" t="n">
-        <v>0.6984126984126985</v>
+        <v>0.6929133858267715</v>
       </c>
       <c r="F87" t="n">
         <v>44</v>
       </c>
       <c r="G87" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H87" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I87" t="n">
         <v>33</v>
@@ -11533,25 +11533,25 @@
         <v>150</v>
       </c>
       <c r="B91" t="n">
-        <v>0.72</v>
+        <v>0.7066666666666667</v>
       </c>
       <c r="C91" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8113207547169812</v>
       </c>
       <c r="D91" t="n">
         <v>0.5584415584415584</v>
       </c>
       <c r="E91" t="n">
-        <v>0.671875</v>
+        <v>0.6615384615384615</v>
       </c>
       <c r="F91" t="n">
         <v>43</v>
       </c>
       <c r="G91" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H91" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I91" t="n">
         <v>34</v>
@@ -11627,19 +11627,19 @@
         <v>150</v>
       </c>
       <c r="B93" t="n">
-        <v>0.7133333333333334</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="C93" t="n">
-        <v>0.9516129032258065</v>
+        <v>0.9538461538461539</v>
       </c>
       <c r="D93" t="n">
-        <v>0.5959595959595959</v>
+        <v>0.6262626262626263</v>
       </c>
       <c r="E93" t="n">
-        <v>0.732919254658385</v>
+        <v>0.7560975609756098</v>
       </c>
       <c r="F93" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G93" t="n">
         <v>48</v>
@@ -11648,7 +11648,7 @@
         <v>3</v>
       </c>
       <c r="I93" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -12003,25 +12003,25 @@
         <v>150</v>
       </c>
       <c r="B101" t="n">
-        <v>0.78</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="C101" t="n">
-        <v>0.5957446808510638</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="D101" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="E101" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.6363636363636365</v>
       </c>
       <c r="F101" t="n">
         <v>28</v>
       </c>
       <c r="G101" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H101" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I101" t="n">
         <v>14</v>
@@ -12050,25 +12050,25 @@
         <v>150</v>
       </c>
       <c r="B102" t="n">
-        <v>0.82</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C102" t="n">
-        <v>0.6229508196721312</v>
+        <v>0.6440677966101694</v>
       </c>
       <c r="D102" t="n">
         <v>0.9047619047619048</v>
       </c>
       <c r="E102" t="n">
-        <v>0.7378640776699029</v>
+        <v>0.7524752475247525</v>
       </c>
       <c r="F102" t="n">
         <v>38</v>
       </c>
       <c r="G102" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H102" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I102" t="n">
         <v>4</v>
@@ -12332,25 +12332,25 @@
         <v>150</v>
       </c>
       <c r="B108" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="C108" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D108" t="n">
         <v>0.6190476190476191</v>
       </c>
       <c r="E108" t="n">
-        <v>0.6500000000000001</v>
+        <v>0.6419753086419754</v>
       </c>
       <c r="F108" t="n">
         <v>26</v>
       </c>
       <c r="G108" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H108" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I108" t="n">
         <v>16</v>
@@ -12379,25 +12379,25 @@
         <v>150</v>
       </c>
       <c r="B109" t="n">
-        <v>0.7066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="C109" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="D109" t="n">
         <v>0.8571428571428571</v>
       </c>
       <c r="E109" t="n">
-        <v>0.6206896551724138</v>
+        <v>0.6</v>
       </c>
       <c r="F109" t="n">
         <v>36</v>
       </c>
       <c r="G109" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H109" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I109" t="n">
         <v>6</v>
@@ -12614,25 +12614,25 @@
         <v>150</v>
       </c>
       <c r="B114" t="n">
-        <v>0.9466666666666667</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C114" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.6842105263157895</v>
       </c>
       <c r="D114" t="n">
         <v>0.8125</v>
       </c>
       <c r="E114" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.742857142857143</v>
       </c>
       <c r="F114" t="n">
         <v>13</v>
       </c>
       <c r="G114" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I114" t="n">
         <v>3</v>
@@ -12802,25 +12802,25 @@
         <v>150</v>
       </c>
       <c r="B118" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.9</v>
       </c>
       <c r="C118" t="n">
-        <v>0.5357142857142857</v>
+        <v>0.5172413793103449</v>
       </c>
       <c r="D118" t="n">
         <v>0.9375</v>
       </c>
       <c r="E118" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="F118" t="n">
         <v>15</v>
       </c>
       <c r="G118" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H118" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I118" t="n">
         <v>1</v>
@@ -12849,25 +12849,25 @@
         <v>150</v>
       </c>
       <c r="B119" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.7933333333333333</v>
       </c>
       <c r="C119" t="n">
-        <v>0.7068965517241379</v>
+        <v>0.7454545454545455</v>
       </c>
       <c r="D119" t="n">
         <v>0.7068965517241379</v>
       </c>
       <c r="E119" t="n">
-        <v>0.7068965517241379</v>
+        <v>0.7256637168141592</v>
       </c>
       <c r="F119" t="n">
         <v>41</v>
       </c>
       <c r="G119" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H119" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I119" t="n">
         <v>17</v>
@@ -12899,25 +12899,25 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C120" t="n">
-        <v>0.72</v>
+        <v>0.726027397260274</v>
       </c>
       <c r="D120" t="n">
-        <v>0.9310344827586207</v>
+        <v>0.9137931034482759</v>
       </c>
       <c r="E120" t="n">
-        <v>0.8120300751879699</v>
+        <v>0.8091603053435115</v>
       </c>
       <c r="F120" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G120" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H120" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I120" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -13178,25 +13178,25 @@
         <v>150</v>
       </c>
       <c r="B126" t="n">
-        <v>0.7866666666666666</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="C126" t="n">
-        <v>0.75</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="D126" t="n">
         <v>0.6724137931034483</v>
       </c>
       <c r="E126" t="n">
-        <v>0.709090909090909</v>
+        <v>0.6964285714285714</v>
       </c>
       <c r="F126" t="n">
         <v>39</v>
       </c>
       <c r="G126" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H126" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I126" t="n">
         <v>19</v>
@@ -13225,28 +13225,28 @@
         <v>150</v>
       </c>
       <c r="B127" t="n">
-        <v>0.62</v>
+        <v>0.6066666666666667</v>
       </c>
       <c r="C127" t="n">
-        <v>0.504950495049505</v>
+        <v>0.4952380952380953</v>
       </c>
       <c r="D127" t="n">
-        <v>0.8793103448275862</v>
+        <v>0.896551724137931</v>
       </c>
       <c r="E127" t="n">
-        <v>0.6415094339622641</v>
+        <v>0.6380368098159509</v>
       </c>
       <c r="F127" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G127" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H127" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I127" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -13319,25 +13319,25 @@
         <v>150</v>
       </c>
       <c r="B129" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.7133333333333334</v>
       </c>
       <c r="C129" t="n">
-        <v>0.7547169811320755</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D129" t="n">
         <v>0.5970149253731343</v>
       </c>
       <c r="E129" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6504065040650405</v>
       </c>
       <c r="F129" t="n">
         <v>40</v>
       </c>
       <c r="G129" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H129" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I129" t="n">
         <v>27</v>
@@ -13413,25 +13413,25 @@
         <v>150</v>
       </c>
       <c r="B131" t="n">
-        <v>0.4066666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="C131" t="n">
-        <v>0.392156862745098</v>
+        <v>0.3883495145631068</v>
       </c>
       <c r="D131" t="n">
         <v>0.5970149253731343</v>
       </c>
       <c r="E131" t="n">
-        <v>0.4733727810650887</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="F131" t="n">
         <v>40</v>
       </c>
       <c r="G131" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H131" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I131" t="n">
         <v>27</v>
@@ -13460,25 +13460,25 @@
         <v>150</v>
       </c>
       <c r="B132" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.62</v>
       </c>
       <c r="C132" t="n">
-        <v>0.84</v>
+        <v>0.65625</v>
       </c>
       <c r="D132" t="n">
         <v>0.3134328358208955</v>
       </c>
       <c r="E132" t="n">
-        <v>0.4565217391304348</v>
+        <v>0.4242424242424243</v>
       </c>
       <c r="F132" t="n">
         <v>21</v>
       </c>
       <c r="G132" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="H132" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I132" t="n">
         <v>46</v>
@@ -13648,25 +13648,25 @@
         <v>150</v>
       </c>
       <c r="B136" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5266666666666666</v>
       </c>
       <c r="C136" t="n">
-        <v>0.4805194805194805</v>
+        <v>0.4743589743589743</v>
       </c>
       <c r="D136" t="n">
         <v>0.5522388059701493</v>
       </c>
       <c r="E136" t="n">
-        <v>0.5138888888888888</v>
+        <v>0.5103448275862068</v>
       </c>
       <c r="F136" t="n">
         <v>37</v>
       </c>
       <c r="G136" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H136" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I136" t="n">
         <v>30</v>
@@ -13698,25 +13698,25 @@
         <v>0.6066666666666667</v>
       </c>
       <c r="C137" t="n">
-        <v>0.5102040816326531</v>
+        <v>0.5098039215686274</v>
       </c>
       <c r="D137" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="E137" t="n">
-        <v>0.4587155963302753</v>
+        <v>0.4684684684684685</v>
       </c>
       <c r="F137" t="n">
+        <v>26</v>
+      </c>
+      <c r="G137" t="n">
+        <v>65</v>
+      </c>
+      <c r="H137" t="n">
         <v>25</v>
       </c>
-      <c r="G137" t="n">
-        <v>66</v>
-      </c>
-      <c r="H137" t="n">
-        <v>24</v>
-      </c>
       <c r="I137" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
@@ -13742,25 +13742,25 @@
         <v>150</v>
       </c>
       <c r="B138" t="n">
-        <v>0.7533333333333333</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="C138" t="n">
-        <v>0.7346938775510204</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="D138" t="n">
         <v>0.6</v>
       </c>
       <c r="E138" t="n">
-        <v>0.6605504587155964</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F138" t="n">
         <v>36</v>
       </c>
       <c r="G138" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H138" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I138" t="n">
         <v>24</v>
@@ -13836,25 +13836,25 @@
         <v>150</v>
       </c>
       <c r="B140" t="n">
-        <v>0.3466666666666667</v>
+        <v>0.34</v>
       </c>
       <c r="C140" t="n">
-        <v>0.2934782608695652</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="D140" t="n">
         <v>0.45</v>
       </c>
       <c r="E140" t="n">
-        <v>0.3552631578947368</v>
+        <v>0.3529411764705882</v>
       </c>
       <c r="F140" t="n">
         <v>27</v>
       </c>
       <c r="G140" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H140" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I140" t="n">
         <v>33</v>
@@ -14074,25 +14074,25 @@
         <v>0.52</v>
       </c>
       <c r="C145" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D145" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.35</v>
       </c>
       <c r="E145" t="n">
-        <v>0.3571428571428571</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="F145" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G145" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H145" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I145" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J145" t="inlineStr">
         <is>

</xml_diff>